<commit_message>
percentage rate and photocopy action buttons
</commit_message>
<xml_diff>
--- a/data/import/ANNEX.xlsx
+++ b/data/import/ANNEX.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD9C543-116A-4FF9-BD77-291DD2AAC994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FD652A-C4E7-49D7-8A37-4D47F8CD2A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BAC" sheetId="2" r:id="rId1"/>
@@ -13,13 +13,17 @@
     <sheet name="4AM" sheetId="3" r:id="rId3"/>
     <sheet name="3AM" sheetId="6" r:id="rId4"/>
     <sheet name="2AM" sheetId="7" r:id="rId5"/>
+    <sheet name="1AM" sheetId="8" r:id="rId6"/>
+    <sheet name="5AP" sheetId="9" r:id="rId7"/>
+    <sheet name="4AP" sheetId="10" r:id="rId8"/>
+    <sheet name="3AP" sheetId="11" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="656">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1469" uniqueCount="785">
   <si>
     <t>الاسم واللقب</t>
   </si>
@@ -1987,6 +1991,393 @@
   </si>
   <si>
     <t>BON08(06/10/2026)</t>
+  </si>
+  <si>
+    <t>عميرش 1AM</t>
+  </si>
+  <si>
+    <t>حركاتي جواد</t>
+  </si>
+  <si>
+    <t>BON04(06/10/2026)</t>
+  </si>
+  <si>
+    <t>بن هلال ياسمين</t>
+  </si>
+  <si>
+    <t>BON02(06/10/2026)</t>
+  </si>
+  <si>
+    <t>بن عزوز 1 متوسط</t>
+  </si>
+  <si>
+    <t>حيمد محمد مهدي</t>
+  </si>
+  <si>
+    <t>07 70243227</t>
+  </si>
+  <si>
+    <t>BON01(01/10/2026)</t>
+  </si>
+  <si>
+    <t>5 ابتدائي رياضيات</t>
+  </si>
+  <si>
+    <t>الكنز لجين</t>
+  </si>
+  <si>
+    <t>06 60 51 31 68</t>
+  </si>
+  <si>
+    <t>BON 01(17/08/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">يزيد خليل </t>
+  </si>
+  <si>
+    <t>0798 72 14 00/0782 86 30 88</t>
+  </si>
+  <si>
+    <t>BON 02(07/09/2026)</t>
+  </si>
+  <si>
+    <t>BON 12(18/09/2026)</t>
+  </si>
+  <si>
+    <t>بومحراث جينان مارية</t>
+  </si>
+  <si>
+    <t>BON 04(15/09/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">بلزرق يوسف </t>
+  </si>
+  <si>
+    <t>BON 05(15/09/2026)</t>
+  </si>
+  <si>
+    <t>بوالحوت امجد</t>
+  </si>
+  <si>
+    <t>BON 06(16/09/2026)</t>
+  </si>
+  <si>
+    <t>بوالقرع ميلسا</t>
+  </si>
+  <si>
+    <t>07 70340943/07 74717459</t>
+  </si>
+  <si>
+    <t>BON 07(18/09/2026)</t>
+  </si>
+  <si>
+    <t>حمادي سجود</t>
+  </si>
+  <si>
+    <t>BON 08(18/09/2026)</t>
+  </si>
+  <si>
+    <t>قلي محمد</t>
+  </si>
+  <si>
+    <t>BON 09(18/09/2026)</t>
+  </si>
+  <si>
+    <t>غولة ميراس</t>
+  </si>
+  <si>
+    <t>BON11(18/09/2026)</t>
+  </si>
+  <si>
+    <t>معمري ميسم</t>
+  </si>
+  <si>
+    <t>BON13(18/09/2026)</t>
+  </si>
+  <si>
+    <t>زغدود مبارك طهى</t>
+  </si>
+  <si>
+    <t>06 70187705/06 58614129</t>
+  </si>
+  <si>
+    <t>BON14(18/09/2026)</t>
+  </si>
+  <si>
+    <t>مشارة يوسف</t>
+  </si>
+  <si>
+    <t>BON21(18/09/2026)</t>
+  </si>
+  <si>
+    <t>شرقي محمد رائد</t>
+  </si>
+  <si>
+    <t>BON22(24/09/2026)</t>
+  </si>
+  <si>
+    <t>بوحلاس رحمة اميمة</t>
+  </si>
+  <si>
+    <t>BON23(24/09/2026)</t>
+  </si>
+  <si>
+    <t>جعوط تسنيم</t>
+  </si>
+  <si>
+    <t>BON 24(25/09/2026)</t>
+  </si>
+  <si>
+    <t>BON 31(02/10/2026)</t>
+  </si>
+  <si>
+    <t>عبد الرزاق اسلام</t>
+  </si>
+  <si>
+    <t>BON 29(02/10/2026)</t>
+  </si>
+  <si>
+    <t>محتوم جود</t>
+  </si>
+  <si>
+    <t>BON 30(02/10/2026)</t>
+  </si>
+  <si>
+    <t>لبيض اياد</t>
+  </si>
+  <si>
+    <t>BON 32(02/10/2026)</t>
+  </si>
+  <si>
+    <t>5 ابتدائي لغة عربية</t>
+  </si>
+  <si>
+    <t>لبيض اياد امجد</t>
+  </si>
+  <si>
+    <t>0554 01 09 35/0550 96 92 60</t>
+  </si>
+  <si>
+    <t>0656 25 12 40</t>
+  </si>
+  <si>
+    <t>0776 62 30 59/0781 57 01 21</t>
+  </si>
+  <si>
+    <t>0672 52 80 97</t>
+  </si>
+  <si>
+    <t>0673 53 59 18/0668 25 72 81</t>
+  </si>
+  <si>
+    <t>0659 17 24 43/0779 83 87 06</t>
+  </si>
+  <si>
+    <t>BON 02(17/09/2026)</t>
+  </si>
+  <si>
+    <t>BON 11(18/09/2026)</t>
+  </si>
+  <si>
+    <t>BON 13(18/09/2026)</t>
+  </si>
+  <si>
+    <t>BON 14(18/09/2026)</t>
+  </si>
+  <si>
+    <t>BON24(22/09/2026)</t>
+  </si>
+  <si>
+    <t>BON 34(02/10/2026)</t>
+  </si>
+  <si>
+    <t>بن عزوز 5 ابتدائي</t>
+  </si>
+  <si>
+    <t>BON 10(18/08/2026)</t>
+  </si>
+  <si>
+    <t>تليلي دعاء</t>
+  </si>
+  <si>
+    <t>0791 44 05 20/0699 66 11 14</t>
+  </si>
+  <si>
+    <t>BON 26(26/09/2026)</t>
+  </si>
+  <si>
+    <t>عليوة فادي</t>
+  </si>
+  <si>
+    <t>BON 27(26/09/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عمير  عبد المهيمن </t>
+  </si>
+  <si>
+    <t>BON 28(29/09/2026)</t>
+  </si>
+  <si>
+    <t>بوديدة عبد السلام</t>
+  </si>
+  <si>
+    <t>BON 33(02/10/2026)</t>
+  </si>
+  <si>
+    <t>BON 35(02/10/2026)</t>
+  </si>
+  <si>
+    <t>شريبي لجين</t>
+  </si>
+  <si>
+    <t>BON 36(03/10/2026)</t>
+  </si>
+  <si>
+    <t>مروة 5 ابتدائي</t>
+  </si>
+  <si>
+    <t>يزيد خليل</t>
+  </si>
+  <si>
+    <t>BON 38(04/10/2026)</t>
+  </si>
+  <si>
+    <t>BON 10(18/09/2026)</t>
+  </si>
+  <si>
+    <t>جعطوط تسنيم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تليلي دعاء </t>
+  </si>
+  <si>
+    <t>BON37(4/10/2026)</t>
+  </si>
+  <si>
+    <t>مروك ادم</t>
+  </si>
+  <si>
+    <t>BON39(4/10/2026)</t>
+  </si>
+  <si>
+    <t>4 ابتدائي لغة عربية</t>
+  </si>
+  <si>
+    <t>حيمد أمير</t>
+  </si>
+  <si>
+    <t>BON 52/3as(07/09/2026)</t>
+  </si>
+  <si>
+    <t>بوبكر عبد الرحمان</t>
+  </si>
+  <si>
+    <t>BON 53/3as(07/09/2026)</t>
+  </si>
+  <si>
+    <t>بوحلاسة مجيب الرحمان</t>
+  </si>
+  <si>
+    <t>BON 54/3as(07/09/2026)</t>
+  </si>
+  <si>
+    <t>زردازي عبد الودود</t>
+  </si>
+  <si>
+    <t>BON 01(19/09/2026)</t>
+  </si>
+  <si>
+    <t>بوعافي براء</t>
+  </si>
+  <si>
+    <t>06 99753989</t>
+  </si>
+  <si>
+    <t>BON 02(22/09/2026)</t>
+  </si>
+  <si>
+    <t>بن محمد ياسر</t>
+  </si>
+  <si>
+    <t>BON 03(25/09/2026)</t>
+  </si>
+  <si>
+    <t>ومان نيزار</t>
+  </si>
+  <si>
+    <t>05 60908908</t>
+  </si>
+  <si>
+    <t>BON 05(25/09/2026)</t>
+  </si>
+  <si>
+    <t>حركات تيم</t>
+  </si>
+  <si>
+    <t>BON 07(02/10/2026)</t>
+  </si>
+  <si>
+    <t>بن فطيمة يحي وليد</t>
+  </si>
+  <si>
+    <t>BON 08(02/10/2026)</t>
+  </si>
+  <si>
+    <t>فيلالي جوري أسماء</t>
+  </si>
+  <si>
+    <t>BON 09(02/10/2026)</t>
+  </si>
+  <si>
+    <t>غراب ياسمين</t>
+  </si>
+  <si>
+    <t>BON 10(02/10/2026)</t>
+  </si>
+  <si>
+    <t>4 ابتدائي رياضيات</t>
+  </si>
+  <si>
+    <t>بن عزوز 4 ابتدائي</t>
+  </si>
+  <si>
+    <t>BON02(22/092026)</t>
+  </si>
+  <si>
+    <t>BON04(25/092026)</t>
+  </si>
+  <si>
+    <t>نموشي مريم جنى</t>
+  </si>
+  <si>
+    <t>BON 06(30/09/2026)</t>
+  </si>
+  <si>
+    <t>3 ابتدائي لغة عربية</t>
+  </si>
+  <si>
+    <t>بركان بهاء الدين</t>
+  </si>
+  <si>
+    <t>بيدي يحي احمد</t>
+  </si>
+  <si>
+    <t>BON 02(21/09/2026)</t>
+  </si>
+  <si>
+    <t>دولة انس نجم الدين</t>
+  </si>
+  <si>
+    <t>BON 03(02/10/2026)</t>
+  </si>
+  <si>
+    <t>بوفندي محمد الإسلام</t>
+  </si>
+  <si>
+    <t>BON 04(02/10/2026)</t>
+  </si>
+  <si>
+    <t>3 ابتدائي رياضيات</t>
   </si>
 </sst>
 </file>
@@ -12635,4 +13026,3230 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C6C7AE0-3130-40DD-BF4E-D974E3CC618F}">
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="16"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+    </row>
+    <row r="2" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>656</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="19"/>
+    </row>
+    <row r="3" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>657</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="7">
+        <v>250</v>
+      </c>
+      <c r="D4" s="7">
+        <v>1500</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>659</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="13">
+        <v>250</v>
+      </c>
+      <c r="D6" s="13">
+        <v>1500</v>
+      </c>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10" t="s">
+        <v>660</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>660</v>
+      </c>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+    </row>
+    <row r="11" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="17" t="s">
+        <v>661</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="19"/>
+    </row>
+    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="20" t="s">
+        <v>662</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="C13" s="7">
+        <v>250</v>
+      </c>
+      <c r="D13" s="7">
+        <v>1500</v>
+      </c>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="15"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="10" t="s">
+        <v>664</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>664</v>
+      </c>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A11:I11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58430E14-9518-4E22-9079-0ACEE1858FC0}">
+  <dimension ref="A1:I117"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.85546875" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="3" max="4" width="20.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="16"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+    </row>
+    <row r="2" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>665</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="19"/>
+    </row>
+    <row r="3" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>669</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>670</v>
+      </c>
+      <c r="C6" s="13">
+        <v>250</v>
+      </c>
+      <c r="D6" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10" t="s">
+        <v>671</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>672</v>
+      </c>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>673</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="13">
+        <v>250</v>
+      </c>
+      <c r="D8" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="10" t="s">
+        <v>674</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>674</v>
+      </c>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>675</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13">
+        <v>250</v>
+      </c>
+      <c r="D10" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="15"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>677</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="13">
+        <v>250</v>
+      </c>
+      <c r="D12" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="15"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="10" t="s">
+        <v>678</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>678</v>
+      </c>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>679</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>680</v>
+      </c>
+      <c r="C14" s="13">
+        <v>250</v>
+      </c>
+      <c r="D14" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="15"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="10" t="s">
+        <v>681</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>681</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>682</v>
+      </c>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13">
+        <v>250</v>
+      </c>
+      <c r="D16" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="10" t="s">
+        <v>683</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>683</v>
+      </c>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>684</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="13">
+        <v>250</v>
+      </c>
+      <c r="D18" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="10" t="s">
+        <v>685</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>685</v>
+      </c>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>686</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="C20" s="13">
+        <v>250</v>
+      </c>
+      <c r="D20" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="15"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="10" t="s">
+        <v>687</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>687</v>
+      </c>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
+        <v>688</v>
+      </c>
+      <c r="B22" s="12"/>
+      <c r="C22" s="13">
+        <v>250</v>
+      </c>
+      <c r="D22" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="15"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="10" t="s">
+        <v>689</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>689</v>
+      </c>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>690</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>691</v>
+      </c>
+      <c r="C24" s="13">
+        <v>250</v>
+      </c>
+      <c r="D24" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="15"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="10" t="s">
+        <v>692</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>692</v>
+      </c>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
+        <v>693</v>
+      </c>
+      <c r="B26" s="12"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="15"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10" t="s">
+        <v>694</v>
+      </c>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
+        <v>695</v>
+      </c>
+      <c r="B28" s="12"/>
+      <c r="C28" s="13">
+        <v>250</v>
+      </c>
+      <c r="D28" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="15"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="10" t="s">
+        <v>696</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>696</v>
+      </c>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
+        <v>697</v>
+      </c>
+      <c r="B30" s="12"/>
+      <c r="C30" s="13">
+        <v>250</v>
+      </c>
+      <c r="D30" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="15"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="10" t="s">
+        <v>698</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>698</v>
+      </c>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="14" t="s">
+        <v>699</v>
+      </c>
+      <c r="B32" s="12"/>
+      <c r="C32" s="13">
+        <v>250</v>
+      </c>
+      <c r="D32" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="15"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="10" t="s">
+        <v>700</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>701</v>
+      </c>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
+        <v>702</v>
+      </c>
+      <c r="B34" s="12"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E34" s="13"/>
+      <c r="F34" s="13"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="15"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10" t="s">
+        <v>703</v>
+      </c>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
+        <v>704</v>
+      </c>
+      <c r="B36" s="12"/>
+      <c r="C36" s="13">
+        <v>250</v>
+      </c>
+      <c r="D36" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="15"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="10" t="s">
+        <v>705</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>705</v>
+      </c>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>706</v>
+      </c>
+      <c r="B38" s="12"/>
+      <c r="C38" s="13">
+        <v>250</v>
+      </c>
+      <c r="D38" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="15"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="10" t="s">
+        <v>707</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>707</v>
+      </c>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="11"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11"/>
+    </row>
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="16"/>
+      <c r="B42" s="16"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16"/>
+      <c r="F42" s="16"/>
+      <c r="G42" s="16"/>
+      <c r="H42" s="16"/>
+      <c r="I42" s="16"/>
+    </row>
+    <row r="43" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="17" t="s">
+        <v>708</v>
+      </c>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
+      <c r="G43" s="18"/>
+      <c r="H43" s="18"/>
+      <c r="I43" s="19"/>
+    </row>
+    <row r="44" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="C45" s="7">
+        <v>250</v>
+      </c>
+      <c r="D45" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="8"/>
+      <c r="H45" s="8"/>
+      <c r="I45" s="8"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="15"/>
+      <c r="B46" s="9"/>
+      <c r="C46" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="11"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="11"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="14" t="s">
+        <v>669</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>437</v>
+      </c>
+      <c r="C47" s="13">
+        <v>250</v>
+      </c>
+      <c r="D47" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E47" s="13"/>
+      <c r="F47" s="13"/>
+      <c r="G47" s="11"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="15"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="10" t="s">
+        <v>716</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>672</v>
+      </c>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="11"/>
+      <c r="H48" s="11"/>
+      <c r="I48" s="11"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="14" t="s">
+        <v>673</v>
+      </c>
+      <c r="B49" s="12" t="s">
+        <v>710</v>
+      </c>
+      <c r="C49" s="13">
+        <v>250</v>
+      </c>
+      <c r="D49" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="11"/>
+      <c r="H49" s="11"/>
+      <c r="I49" s="11"/>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="15"/>
+      <c r="B50" s="9"/>
+      <c r="C50" s="10" t="s">
+        <v>674</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>674</v>
+      </c>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="11"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="14" t="s">
+        <v>675</v>
+      </c>
+      <c r="B51" s="12"/>
+      <c r="C51" s="13">
+        <v>250</v>
+      </c>
+      <c r="D51" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E51" s="13"/>
+      <c r="F51" s="13"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="15"/>
+      <c r="B52" s="9"/>
+      <c r="C52" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="E52" s="10"/>
+      <c r="F52" s="10"/>
+      <c r="G52" s="11"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="14" t="s">
+        <v>677</v>
+      </c>
+      <c r="B53" s="12" t="s">
+        <v>711</v>
+      </c>
+      <c r="C53" s="13">
+        <v>250</v>
+      </c>
+      <c r="D53" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E53" s="13"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="11"/>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="15"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="10" t="s">
+        <v>678</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>678</v>
+      </c>
+      <c r="E54" s="10"/>
+      <c r="F54" s="10"/>
+      <c r="G54" s="11"/>
+      <c r="H54" s="11"/>
+      <c r="I54" s="11"/>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="14" t="s">
+        <v>679</v>
+      </c>
+      <c r="B55" s="12" t="s">
+        <v>680</v>
+      </c>
+      <c r="C55" s="13">
+        <v>250</v>
+      </c>
+      <c r="D55" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E55" s="13"/>
+      <c r="F55" s="13"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="11"/>
+      <c r="I55" s="11"/>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="15"/>
+      <c r="B56" s="9"/>
+      <c r="C56" s="10" t="s">
+        <v>681</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>681</v>
+      </c>
+      <c r="E56" s="10"/>
+      <c r="F56" s="10"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="14" t="s">
+        <v>682</v>
+      </c>
+      <c r="B57" s="12"/>
+      <c r="C57" s="13">
+        <v>250</v>
+      </c>
+      <c r="D57" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11"/>
+      <c r="I57" s="11"/>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="15"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="10" t="s">
+        <v>683</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>683</v>
+      </c>
+      <c r="E58" s="10"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" s="14" t="s">
+        <v>684</v>
+      </c>
+      <c r="B59" s="12"/>
+      <c r="C59" s="13">
+        <v>250</v>
+      </c>
+      <c r="D59" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E59" s="13"/>
+      <c r="F59" s="13"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="15"/>
+      <c r="B60" s="9"/>
+      <c r="C60" s="10" t="s">
+        <v>685</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>685</v>
+      </c>
+      <c r="E60" s="10"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11"/>
+      <c r="I60" s="11"/>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="14" t="s">
+        <v>686</v>
+      </c>
+      <c r="B61" s="12"/>
+      <c r="C61" s="13">
+        <v>250</v>
+      </c>
+      <c r="D61" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E61" s="13"/>
+      <c r="F61" s="13"/>
+      <c r="G61" s="11"/>
+      <c r="H61" s="11"/>
+      <c r="I61" s="11"/>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="15"/>
+      <c r="B62" s="9"/>
+      <c r="C62" s="10" t="s">
+        <v>717</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>717</v>
+      </c>
+      <c r="E62" s="10"/>
+      <c r="F62" s="10"/>
+      <c r="G62" s="11"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="11"/>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="14" t="s">
+        <v>688</v>
+      </c>
+      <c r="B63" s="12" t="s">
+        <v>712</v>
+      </c>
+      <c r="C63" s="13">
+        <v>250</v>
+      </c>
+      <c r="D63" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E63" s="13"/>
+      <c r="F63" s="13"/>
+      <c r="G63" s="11"/>
+      <c r="H63" s="11"/>
+      <c r="I63" s="11"/>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="15"/>
+      <c r="B64" s="9"/>
+      <c r="C64" s="10" t="s">
+        <v>718</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>718</v>
+      </c>
+      <c r="E64" s="10"/>
+      <c r="F64" s="10"/>
+      <c r="G64" s="11"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="11"/>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="14" t="s">
+        <v>690</v>
+      </c>
+      <c r="B65" s="12" t="s">
+        <v>691</v>
+      </c>
+      <c r="C65" s="13">
+        <v>250</v>
+      </c>
+      <c r="D65" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E65" s="13"/>
+      <c r="F65" s="13"/>
+      <c r="G65" s="11"/>
+      <c r="H65" s="11"/>
+      <c r="I65" s="11"/>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="15"/>
+      <c r="B66" s="9"/>
+      <c r="C66" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="D66" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="E66" s="10"/>
+      <c r="F66" s="10"/>
+      <c r="G66" s="11"/>
+      <c r="H66" s="11"/>
+      <c r="I66" s="11"/>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67" s="14" t="s">
+        <v>693</v>
+      </c>
+      <c r="B67" s="12"/>
+      <c r="C67" s="13"/>
+      <c r="D67" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E67" s="13"/>
+      <c r="F67" s="13"/>
+      <c r="G67" s="11"/>
+      <c r="H67" s="11"/>
+      <c r="I67" s="11"/>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="15"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="10" t="s">
+        <v>694</v>
+      </c>
+      <c r="E68" s="10"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="11"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="14" t="s">
+        <v>695</v>
+      </c>
+      <c r="B69" s="12" t="s">
+        <v>713</v>
+      </c>
+      <c r="C69" s="13">
+        <v>250</v>
+      </c>
+      <c r="D69" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E69" s="13"/>
+      <c r="F69" s="13"/>
+      <c r="G69" s="11"/>
+      <c r="H69" s="11"/>
+      <c r="I69" s="11"/>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="15"/>
+      <c r="B70" s="9"/>
+      <c r="C70" s="10" t="s">
+        <v>720</v>
+      </c>
+      <c r="D70" s="10" t="s">
+        <v>720</v>
+      </c>
+      <c r="E70" s="10"/>
+      <c r="F70" s="10"/>
+      <c r="G70" s="11"/>
+      <c r="H70" s="11"/>
+      <c r="I70" s="11"/>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71" s="14" t="s">
+        <v>697</v>
+      </c>
+      <c r="B71" s="12" t="s">
+        <v>714</v>
+      </c>
+      <c r="C71" s="13">
+        <v>250</v>
+      </c>
+      <c r="D71" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E71" s="13"/>
+      <c r="F71" s="13"/>
+      <c r="G71" s="11"/>
+      <c r="H71" s="11"/>
+      <c r="I71" s="11"/>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" s="15"/>
+      <c r="B72" s="9"/>
+      <c r="C72" s="10" t="s">
+        <v>698</v>
+      </c>
+      <c r="D72" s="10" t="s">
+        <v>698</v>
+      </c>
+      <c r="E72" s="10"/>
+      <c r="F72" s="10"/>
+      <c r="G72" s="11"/>
+      <c r="H72" s="11"/>
+      <c r="I72" s="11"/>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" s="14" t="s">
+        <v>699</v>
+      </c>
+      <c r="B73" s="12" t="s">
+        <v>715</v>
+      </c>
+      <c r="C73" s="13">
+        <v>250</v>
+      </c>
+      <c r="D73" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E73" s="13"/>
+      <c r="F73" s="13"/>
+      <c r="G73" s="11"/>
+      <c r="H73" s="11"/>
+      <c r="I73" s="11"/>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A74" s="15"/>
+      <c r="B74" s="9"/>
+      <c r="C74" s="10" t="s">
+        <v>700</v>
+      </c>
+      <c r="D74" s="10" t="s">
+        <v>701</v>
+      </c>
+      <c r="E74" s="10"/>
+      <c r="F74" s="10"/>
+      <c r="G74" s="11"/>
+      <c r="H74" s="11"/>
+      <c r="I74" s="11"/>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A75" s="14" t="s">
+        <v>702</v>
+      </c>
+      <c r="B75" s="12"/>
+      <c r="C75" s="13"/>
+      <c r="D75" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E75" s="13"/>
+      <c r="F75" s="13"/>
+      <c r="G75" s="11"/>
+      <c r="H75" s="11"/>
+      <c r="I75" s="11"/>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76" s="15"/>
+      <c r="B76" s="9"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="10" t="s">
+        <v>703</v>
+      </c>
+      <c r="E76" s="10"/>
+      <c r="F76" s="10"/>
+      <c r="G76" s="11"/>
+      <c r="H76" s="11"/>
+      <c r="I76" s="11"/>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A77" s="14" t="s">
+        <v>709</v>
+      </c>
+      <c r="B77" s="12"/>
+      <c r="C77" s="13">
+        <v>250</v>
+      </c>
+      <c r="D77" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E77" s="13"/>
+      <c r="F77" s="13"/>
+      <c r="G77" s="11"/>
+      <c r="H77" s="11"/>
+      <c r="I77" s="11"/>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A78" s="15"/>
+      <c r="B78" s="9"/>
+      <c r="C78" s="10" t="s">
+        <v>707</v>
+      </c>
+      <c r="D78" s="10" t="s">
+        <v>707</v>
+      </c>
+      <c r="E78" s="10"/>
+      <c r="F78" s="10"/>
+      <c r="G78" s="11"/>
+      <c r="H78" s="11"/>
+      <c r="I78" s="11"/>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A79" s="14" t="s">
+        <v>704</v>
+      </c>
+      <c r="B79" s="12"/>
+      <c r="C79" s="13"/>
+      <c r="D79" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E79" s="13"/>
+      <c r="F79" s="13"/>
+      <c r="G79" s="11"/>
+      <c r="H79" s="11"/>
+      <c r="I79" s="11"/>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A80" s="15"/>
+      <c r="B80" s="9"/>
+      <c r="C80" s="10"/>
+      <c r="D80" s="10" t="s">
+        <v>721</v>
+      </c>
+      <c r="E80" s="10"/>
+      <c r="F80" s="10"/>
+      <c r="G80" s="11"/>
+      <c r="H80" s="11"/>
+      <c r="I80" s="11"/>
+    </row>
+    <row r="82" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="16"/>
+      <c r="B82" s="16"/>
+      <c r="C82" s="16"/>
+      <c r="D82" s="16"/>
+      <c r="E82" s="16"/>
+      <c r="F82" s="16"/>
+      <c r="G82" s="16"/>
+      <c r="H82" s="16"/>
+      <c r="I82" s="16"/>
+    </row>
+    <row r="83" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="17" t="s">
+        <v>722</v>
+      </c>
+      <c r="B83" s="18"/>
+      <c r="C83" s="18"/>
+      <c r="D83" s="18"/>
+      <c r="E83" s="18"/>
+      <c r="F83" s="18"/>
+      <c r="G83" s="18"/>
+      <c r="H83" s="18"/>
+      <c r="I83" s="19"/>
+    </row>
+    <row r="84" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B84" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D84" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F84" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H84" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I84" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A85" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="C85" s="7">
+        <v>250</v>
+      </c>
+      <c r="D85" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E85" s="7"/>
+      <c r="F85" s="7"/>
+      <c r="G85" s="8"/>
+      <c r="H85" s="8"/>
+      <c r="I85" s="8"/>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" s="15"/>
+      <c r="B86" s="9"/>
+      <c r="C86" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="D86" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="E86" s="10"/>
+      <c r="F86" s="10"/>
+      <c r="G86" s="11"/>
+      <c r="H86" s="11"/>
+      <c r="I86" s="11"/>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" s="14" t="s">
+        <v>684</v>
+      </c>
+      <c r="B87" s="12"/>
+      <c r="C87" s="13">
+        <v>250</v>
+      </c>
+      <c r="D87" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E87" s="13"/>
+      <c r="F87" s="13"/>
+      <c r="G87" s="11"/>
+      <c r="H87" s="11"/>
+      <c r="I87" s="11"/>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" s="15"/>
+      <c r="B88" s="9"/>
+      <c r="C88" s="10" t="s">
+        <v>723</v>
+      </c>
+      <c r="D88" s="10" t="s">
+        <v>723</v>
+      </c>
+      <c r="E88" s="10"/>
+      <c r="F88" s="10"/>
+      <c r="G88" s="11"/>
+      <c r="H88" s="11"/>
+      <c r="I88" s="11"/>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" s="14" t="s">
+        <v>724</v>
+      </c>
+      <c r="B89" s="12" t="s">
+        <v>725</v>
+      </c>
+      <c r="C89" s="13">
+        <v>250</v>
+      </c>
+      <c r="D89" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E89" s="13"/>
+      <c r="F89" s="13"/>
+      <c r="G89" s="11"/>
+      <c r="H89" s="11"/>
+      <c r="I89" s="11"/>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" s="15"/>
+      <c r="B90" s="9"/>
+      <c r="C90" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="D90" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="E90" s="10"/>
+      <c r="F90" s="10"/>
+      <c r="G90" s="11"/>
+      <c r="H90" s="11"/>
+      <c r="I90" s="11"/>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" s="14" t="s">
+        <v>727</v>
+      </c>
+      <c r="B91" s="12"/>
+      <c r="C91" s="13">
+        <v>250</v>
+      </c>
+      <c r="D91" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E91" s="13"/>
+      <c r="F91" s="13"/>
+      <c r="G91" s="11"/>
+      <c r="H91" s="11"/>
+      <c r="I91" s="11"/>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" s="15"/>
+      <c r="B92" s="9"/>
+      <c r="C92" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="D92" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="E92" s="10"/>
+      <c r="F92" s="10"/>
+      <c r="G92" s="11"/>
+      <c r="H92" s="11"/>
+      <c r="I92" s="11"/>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" s="14" t="s">
+        <v>729</v>
+      </c>
+      <c r="B93" s="12"/>
+      <c r="C93" s="13">
+        <v>250</v>
+      </c>
+      <c r="D93" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E93" s="13"/>
+      <c r="F93" s="13"/>
+      <c r="G93" s="11"/>
+      <c r="H93" s="11"/>
+      <c r="I93" s="11"/>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" s="15"/>
+      <c r="B94" s="9"/>
+      <c r="C94" s="10" t="s">
+        <v>730</v>
+      </c>
+      <c r="D94" s="10" t="s">
+        <v>730</v>
+      </c>
+      <c r="E94" s="10"/>
+      <c r="F94" s="10"/>
+      <c r="G94" s="11"/>
+      <c r="H94" s="11"/>
+      <c r="I94" s="11"/>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" s="14" t="s">
+        <v>731</v>
+      </c>
+      <c r="B95" s="12"/>
+      <c r="C95" s="13">
+        <v>250</v>
+      </c>
+      <c r="D95" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E95" s="13"/>
+      <c r="F95" s="13"/>
+      <c r="G95" s="11"/>
+      <c r="H95" s="11"/>
+      <c r="I95" s="11"/>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" s="15"/>
+      <c r="B96" s="9"/>
+      <c r="C96" s="10" t="s">
+        <v>732</v>
+      </c>
+      <c r="D96" s="10" t="s">
+        <v>732</v>
+      </c>
+      <c r="E96" s="10"/>
+      <c r="F96" s="10"/>
+      <c r="G96" s="11"/>
+      <c r="H96" s="11"/>
+      <c r="I96" s="11"/>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" s="14" t="s">
+        <v>702</v>
+      </c>
+      <c r="B97" s="12"/>
+      <c r="C97" s="13"/>
+      <c r="D97" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E97" s="13"/>
+      <c r="F97" s="13"/>
+      <c r="G97" s="11"/>
+      <c r="H97" s="11"/>
+      <c r="I97" s="11"/>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" s="15"/>
+      <c r="B98" s="9"/>
+      <c r="C98" s="10"/>
+      <c r="D98" s="10" t="s">
+        <v>733</v>
+      </c>
+      <c r="E98" s="10"/>
+      <c r="F98" s="10"/>
+      <c r="G98" s="11"/>
+      <c r="H98" s="11"/>
+      <c r="I98" s="11"/>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" s="14" t="s">
+        <v>734</v>
+      </c>
+      <c r="B99" s="12"/>
+      <c r="C99" s="13">
+        <v>250</v>
+      </c>
+      <c r="D99" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E99" s="13"/>
+      <c r="F99" s="13"/>
+      <c r="G99" s="11"/>
+      <c r="H99" s="11"/>
+      <c r="I99" s="11"/>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" s="15"/>
+      <c r="B100" s="9"/>
+      <c r="C100" s="10" t="s">
+        <v>735</v>
+      </c>
+      <c r="D100" s="10" t="s">
+        <v>735</v>
+      </c>
+      <c r="E100" s="10"/>
+      <c r="F100" s="10"/>
+      <c r="G100" s="11"/>
+      <c r="H100" s="11"/>
+      <c r="I100" s="11"/>
+    </row>
+    <row r="103" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="16"/>
+      <c r="B103" s="16"/>
+      <c r="C103" s="16"/>
+      <c r="D103" s="16"/>
+      <c r="E103" s="16"/>
+      <c r="F103" s="16"/>
+      <c r="G103" s="16"/>
+      <c r="H103" s="16"/>
+      <c r="I103" s="16"/>
+    </row>
+    <row r="104" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="17" t="s">
+        <v>736</v>
+      </c>
+      <c r="B104" s="18"/>
+      <c r="C104" s="18"/>
+      <c r="D104" s="18"/>
+      <c r="E104" s="18"/>
+      <c r="F104" s="18"/>
+      <c r="G104" s="18"/>
+      <c r="H104" s="18"/>
+      <c r="I104" s="19"/>
+    </row>
+    <row r="105" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C105" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E105" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F105" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G105" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H105" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I105" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="C106" s="7">
+        <v>250</v>
+      </c>
+      <c r="D106" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E106" s="7"/>
+      <c r="F106" s="7"/>
+      <c r="G106" s="8"/>
+      <c r="H106" s="8"/>
+      <c r="I106" s="8"/>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" s="15"/>
+      <c r="B107" s="9"/>
+      <c r="C107" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="D107" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="E107" s="10"/>
+      <c r="F107" s="10"/>
+      <c r="G107" s="11"/>
+      <c r="H107" s="11"/>
+      <c r="I107" s="11"/>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" s="14" t="s">
+        <v>737</v>
+      </c>
+      <c r="B108" s="12" t="s">
+        <v>437</v>
+      </c>
+      <c r="C108" s="13">
+        <v>250</v>
+      </c>
+      <c r="D108" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E108" s="13"/>
+      <c r="F108" s="13"/>
+      <c r="G108" s="11"/>
+      <c r="H108" s="11"/>
+      <c r="I108" s="11"/>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" s="15"/>
+      <c r="B109" s="9"/>
+      <c r="C109" s="10" t="s">
+        <v>671</v>
+      </c>
+      <c r="D109" s="10" t="s">
+        <v>738</v>
+      </c>
+      <c r="E109" s="10"/>
+      <c r="F109" s="10"/>
+      <c r="G109" s="11"/>
+      <c r="H109" s="11"/>
+      <c r="I109" s="11"/>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" s="14" t="s">
+        <v>684</v>
+      </c>
+      <c r="B110" s="12"/>
+      <c r="C110" s="13"/>
+      <c r="D110" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E110" s="13"/>
+      <c r="F110" s="13"/>
+      <c r="G110" s="11"/>
+      <c r="H110" s="11"/>
+      <c r="I110" s="11"/>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" s="15"/>
+      <c r="B111" s="9"/>
+      <c r="C111" s="10"/>
+      <c r="D111" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="E111" s="10"/>
+      <c r="F111" s="10"/>
+      <c r="G111" s="11"/>
+      <c r="H111" s="11"/>
+      <c r="I111" s="11"/>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112" s="14" t="s">
+        <v>740</v>
+      </c>
+      <c r="B112" s="12"/>
+      <c r="C112" s="13">
+        <v>250</v>
+      </c>
+      <c r="D112" s="13"/>
+      <c r="E112" s="13"/>
+      <c r="F112" s="13"/>
+      <c r="G112" s="11"/>
+      <c r="H112" s="11"/>
+      <c r="I112" s="11"/>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" s="15"/>
+      <c r="B113" s="9"/>
+      <c r="C113" s="10" t="s">
+        <v>700</v>
+      </c>
+      <c r="D113" s="10"/>
+      <c r="E113" s="10"/>
+      <c r="F113" s="10"/>
+      <c r="G113" s="11"/>
+      <c r="H113" s="11"/>
+      <c r="I113" s="11"/>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" s="14" t="s">
+        <v>741</v>
+      </c>
+      <c r="B114" s="12"/>
+      <c r="C114" s="13">
+        <v>250</v>
+      </c>
+      <c r="D114" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E114" s="13"/>
+      <c r="F114" s="13"/>
+      <c r="G114" s="11"/>
+      <c r="H114" s="11"/>
+      <c r="I114" s="11"/>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A115" s="15"/>
+      <c r="B115" s="9"/>
+      <c r="C115" s="10" t="s">
+        <v>742</v>
+      </c>
+      <c r="D115" s="10" t="s">
+        <v>742</v>
+      </c>
+      <c r="E115" s="10"/>
+      <c r="F115" s="10"/>
+      <c r="G115" s="11"/>
+      <c r="H115" s="11"/>
+      <c r="I115" s="11"/>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A116" s="14" t="s">
+        <v>743</v>
+      </c>
+      <c r="B116" s="12"/>
+      <c r="C116" s="13">
+        <v>250</v>
+      </c>
+      <c r="D116" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E116" s="13"/>
+      <c r="F116" s="13"/>
+      <c r="G116" s="11"/>
+      <c r="H116" s="11"/>
+      <c r="I116" s="11"/>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A117" s="15"/>
+      <c r="B117" s="9"/>
+      <c r="C117" s="10" t="s">
+        <v>744</v>
+      </c>
+      <c r="D117" s="10" t="s">
+        <v>744</v>
+      </c>
+      <c r="E117" s="10"/>
+      <c r="F117" s="10"/>
+      <c r="G117" s="11"/>
+      <c r="H117" s="11"/>
+      <c r="I117" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="58">
+    <mergeCell ref="A114:A115"/>
+    <mergeCell ref="A116:A117"/>
+    <mergeCell ref="A103:I103"/>
+    <mergeCell ref="A104:I104"/>
+    <mergeCell ref="A106:A107"/>
+    <mergeCell ref="A108:A109"/>
+    <mergeCell ref="A110:A111"/>
+    <mergeCell ref="A112:A113"/>
+    <mergeCell ref="A89:A90"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="A93:A94"/>
+    <mergeCell ref="A95:A96"/>
+    <mergeCell ref="A97:A98"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="A82:I82"/>
+    <mergeCell ref="A83:I83"/>
+    <mergeCell ref="A85:A86"/>
+    <mergeCell ref="A87:A88"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="A67:A68"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="A73:A74"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A42:I42"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BD8F5EC-C24E-492D-897C-0FB9BD38A5F7}">
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="22.140625" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="16"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+    </row>
+    <row r="2" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>745</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="19"/>
+    </row>
+    <row r="3" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>746</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="7">
+        <v>250</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10" t="s">
+        <v>747</v>
+      </c>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>748</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="13">
+        <v>250</v>
+      </c>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10" t="s">
+        <v>749</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>750</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="13">
+        <v>250</v>
+      </c>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="10" t="s">
+        <v>751</v>
+      </c>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>752</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13">
+        <v>250</v>
+      </c>
+      <c r="D10" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="15"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="10" t="s">
+        <v>753</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>753</v>
+      </c>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>754</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>755</v>
+      </c>
+      <c r="C12" s="13">
+        <v>250</v>
+      </c>
+      <c r="D12" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="15"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="10" t="s">
+        <v>756</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>756</v>
+      </c>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>757</v>
+      </c>
+      <c r="B14" s="12"/>
+      <c r="C14" s="13">
+        <v>250</v>
+      </c>
+      <c r="D14" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="15"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="10" t="s">
+        <v>758</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>758</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>759</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>760</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10" t="s">
+        <v>761</v>
+      </c>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>762</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10" t="s">
+        <v>763</v>
+      </c>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>764</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="C20" s="13">
+        <v>250</v>
+      </c>
+      <c r="D20" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="15"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="10" t="s">
+        <v>765</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>765</v>
+      </c>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
+        <v>766</v>
+      </c>
+      <c r="B22" s="12"/>
+      <c r="C22" s="13">
+        <v>250</v>
+      </c>
+      <c r="D22" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="15"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="10" t="s">
+        <v>767</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>767</v>
+      </c>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>768</v>
+      </c>
+      <c r="B24" s="12"/>
+      <c r="C24" s="13">
+        <v>250</v>
+      </c>
+      <c r="D24" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="15"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="10" t="s">
+        <v>769</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>769</v>
+      </c>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="16"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+    </row>
+    <row r="29" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="17" t="s">
+        <v>770</v>
+      </c>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18"/>
+      <c r="I29" s="19"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="20" t="s">
+        <v>752</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="7">
+        <v>250</v>
+      </c>
+      <c r="D31" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="15"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="10" t="s">
+        <v>753</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>753</v>
+      </c>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="14" t="s">
+        <v>754</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>755</v>
+      </c>
+      <c r="C33" s="13">
+        <v>250</v>
+      </c>
+      <c r="D33" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="15"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="10" t="s">
+        <v>756</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>756</v>
+      </c>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
+        <v>757</v>
+      </c>
+      <c r="B35" s="12"/>
+      <c r="C35" s="13">
+        <v>250</v>
+      </c>
+      <c r="D35" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="15"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="10" t="s">
+        <v>758</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>758</v>
+      </c>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="14" t="s">
+        <v>762</v>
+      </c>
+      <c r="B37" s="12"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="15"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10" t="s">
+        <v>763</v>
+      </c>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="14" t="s">
+        <v>764</v>
+      </c>
+      <c r="B39" s="12"/>
+      <c r="C39" s="13">
+        <v>250</v>
+      </c>
+      <c r="D39" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="11"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="15"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="10" t="s">
+        <v>765</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>765</v>
+      </c>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+    </row>
+    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="16"/>
+      <c r="B43" s="16"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="16"/>
+      <c r="G43" s="16"/>
+      <c r="H43" s="16"/>
+      <c r="I43" s="16"/>
+    </row>
+    <row r="44" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="19"/>
+    </row>
+    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="20" t="s">
+        <v>754</v>
+      </c>
+      <c r="B46" s="6"/>
+      <c r="C46" s="7">
+        <v>250</v>
+      </c>
+      <c r="D46" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="8"/>
+      <c r="I46" s="8"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="15"/>
+      <c r="B47" s="9"/>
+      <c r="C47" s="10" t="s">
+        <v>772</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>772</v>
+      </c>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="11"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="14" t="s">
+        <v>757</v>
+      </c>
+      <c r="B48" s="12"/>
+      <c r="C48" s="13">
+        <v>250</v>
+      </c>
+      <c r="D48" s="13"/>
+      <c r="E48" s="13"/>
+      <c r="F48" s="13"/>
+      <c r="G48" s="11"/>
+      <c r="H48" s="11"/>
+      <c r="I48" s="11"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="15"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="10" t="s">
+        <v>773</v>
+      </c>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="11"/>
+      <c r="H49" s="11"/>
+      <c r="I49" s="11"/>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="14" t="s">
+        <v>774</v>
+      </c>
+      <c r="B50" s="12"/>
+      <c r="C50" s="13">
+        <v>250</v>
+      </c>
+      <c r="D50" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="11"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="15"/>
+      <c r="B51" s="9"/>
+      <c r="C51" s="10" t="s">
+        <v>775</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>775</v>
+      </c>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85925C9E-4B5B-4B50-A16D-F247EAB10B79}">
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.28515625" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" customWidth="1"/>
+    <col min="4" max="4" width="27.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="16"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+    </row>
+    <row r="2" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>776</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="19"/>
+    </row>
+    <row r="3" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>777</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="7">
+        <v>250</v>
+      </c>
+      <c r="D4" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10" t="s">
+        <v>631</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>631</v>
+      </c>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>778</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10" t="s">
+        <v>779</v>
+      </c>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>780</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="13">
+        <v>250</v>
+      </c>
+      <c r="D8" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="10" t="s">
+        <v>781</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>781</v>
+      </c>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>782</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13">
+        <v>250</v>
+      </c>
+      <c r="D10" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="15"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="10" t="s">
+        <v>783</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>783</v>
+      </c>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+    </row>
+    <row r="15" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="17" t="s">
+        <v>784</v>
+      </c>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="19"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="20" t="s">
+        <v>777</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="7">
+        <v>250</v>
+      </c>
+      <c r="D17" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="15"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="10" t="s">
+        <v>631</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>631</v>
+      </c>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
+        <v>778</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="13">
+        <v>250</v>
+      </c>
+      <c r="D19" s="13">
+        <v>1200</v>
+      </c>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="15"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="10" t="s">
+        <v>779</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>779</v>
+      </c>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>